<commit_message>
Add multi-layered TOPSIS recommendation
</commit_message>
<xml_diff>
--- a/outputs/comparison.xlsx
+++ b/outputs/comparison.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,41 +425,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>algorithm</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>top_provider</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>top_score</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>execution_seconds</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>memory_bytes</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>provider_count</t>
         </is>
@@ -468,10 +480,10 @@
         <v>0.74945991265</v>
       </c>
       <c r="D2" t="n">
-        <v>0.005256599994027056</v>
+        <v>0.008813399996142834</v>
       </c>
       <c r="E2" t="n">
-        <v>13208</v>
+        <v>13200</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -483,7 +495,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TOPSIS</t>
+          <t>M-TOPSIS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -492,13 +504,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.695904436185</v>
+        <v>0.762618230264</v>
       </c>
       <c r="D3" t="n">
-        <v>0.08701759998803027</v>
+        <v>0.2505738000036217</v>
       </c>
       <c r="E3" t="n">
-        <v>2569503</v>
+        <v>3222323</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -510,7 +522,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AHP</t>
+          <t>TOPSIS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -519,13 +531,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.74945991265</v>
+        <v>0.695904436185</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0336863000120502</v>
+        <v>0.155110300052911</v>
       </c>
       <c r="E4" t="n">
-        <v>2478807</v>
+        <v>3273786</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
@@ -537,22 +549,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>VIKOR</t>
+          <t>AHP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RetHeaderService</t>
+          <t>dConverterSOAP</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.907956273826</v>
+        <v>0.74945991265</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1933869000058621</v>
+        <v>0.08213720005005598</v>
       </c>
       <c r="E5" t="n">
-        <v>2481063</v>
+        <v>3258025</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -564,22 +576,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PROMETHEE II</t>
+          <t>VIKOR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>dConverterSOAP</t>
+          <t>RetHeaderService</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.74945991265</v>
+        <v>0.907956273826</v>
       </c>
       <c r="D6" t="n">
-        <v>0.03967850000481121</v>
+        <v>0.4496897999779321</v>
       </c>
       <c r="E6" t="n">
-        <v>2478791</v>
+        <v>3261301</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
@@ -591,7 +603,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ELECTRE</t>
+          <t>PROMETHEE II</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -603,10 +615,10 @@
         <v>0.74945991265</v>
       </c>
       <c r="D7" t="n">
-        <v>0.03187550000438932</v>
+        <v>0.09371449996251613</v>
       </c>
       <c r="E7" t="n">
-        <v>2570839</v>
+        <v>3256619</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
@@ -618,7 +630,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAW</t>
+          <t>ELECTRE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -630,10 +642,10 @@
         <v>0.74945991265</v>
       </c>
       <c r="D8" t="n">
-        <v>0.02994580000813585</v>
+        <v>0.05294470000080764</v>
       </c>
       <c r="E8" t="n">
-        <v>2478655</v>
+        <v>3256451</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
@@ -645,27 +657,54 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>SAW</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>dConverterSOAP</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.74945991265</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.04902629996649921</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3256619</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1643</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Weighted Product Model</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>RetHeaderService</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C10" t="n">
         <v>0.553093686444</v>
       </c>
-      <c r="D9" t="n">
-        <v>0.03252369999245275</v>
-      </c>
-      <c r="E9" t="n">
-        <v>2478783</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="n">
+      <c r="D10" t="n">
+        <v>0.09689500002423301</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3258116</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
         <v>1643</v>
       </c>
     </row>

</xml_diff>